<commit_message>
phase final table and ranking
</commit_message>
<xml_diff>
--- a/runapp/www/scores.xlsx
+++ b/runapp/www/scores.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loicl\OneDrive\Documents\Loïc\Divers_non_disque\Data_science\Projet\MesProjets\Coude_du_monde_2026\runapp\www\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loicl\OneDrive\Documents\Loïc\Divers_non_disque\Data_science\Projet\MesProjets\Coupe_du_monde_2026\runapp\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC29929-BE88-4B84-AD1B-A404BFD2345B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E44E9454-DB1C-4C44-89F0-0F85EC29BC60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-4155" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -301,9 +301,6 @@
     <t>Portugal</t>
   </si>
   <si>
-    <t>République Démocratique du Congo</t>
-  </si>
-  <si>
     <t>66457030</t>
   </si>
   <si>
@@ -434,6 +431,9 @@
   </si>
   <si>
     <t>away</t>
+  </si>
+  <si>
+    <t>RD Congo</t>
   </si>
 </sst>
 </file>
@@ -477,7 +477,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -486,6 +486,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -796,28 +802,28 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="3"/>
-    <col min="2" max="2" width="19.88671875" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.44140625" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>123</v>
-      </c>
       <c r="E1" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
@@ -825,15 +831,15 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3">
-        <v>3</v>
-      </c>
-      <c r="D2" s="3">
+      <c r="C2" s="5">
+        <v>3</v>
+      </c>
+      <c r="D2" s="5">
         <v>0</v>
       </c>
       <c r="E2" t="s">
@@ -845,15 +851,15 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="3">
-        <v>2</v>
-      </c>
-      <c r="D3" s="3">
+      <c r="C3" s="5">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5">
         <v>0</v>
       </c>
       <c r="E3" t="s">
@@ -865,15 +871,15 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3">
-        <v>3</v>
-      </c>
-      <c r="D4" s="3">
+      <c r="C4" s="5">
+        <v>3</v>
+      </c>
+      <c r="D4" s="5">
         <v>0</v>
       </c>
       <c r="E4" t="s">
@@ -885,15 +891,15 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="5">
         <v>1</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="5">
         <v>0</v>
       </c>
       <c r="E5" t="s">
@@ -905,15 +911,15 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="5">
         <v>0</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="5">
         <v>3</v>
       </c>
       <c r="E6" t="s">
@@ -925,15 +931,15 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B7" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="5">
         <v>0</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="5">
         <v>2</v>
       </c>
       <c r="E7" t="s">
@@ -945,15 +951,15 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="5">
         <v>0</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="5">
         <v>2</v>
       </c>
       <c r="E8" t="s">
@@ -965,15 +971,15 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B9" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="3">
-        <v>2</v>
-      </c>
-      <c r="D9" s="3">
+      <c r="C9" s="5">
+        <v>2</v>
+      </c>
+      <c r="D9" s="5">
         <v>2</v>
       </c>
       <c r="E9" t="s">
@@ -985,15 +991,15 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B10" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="5">
         <v>0</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="5">
         <v>1</v>
       </c>
       <c r="E10" t="s">
@@ -1005,15 +1011,15 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B11" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="3">
-        <v>2</v>
-      </c>
-      <c r="D11" s="3">
+      <c r="C11" s="5">
+        <v>2</v>
+      </c>
+      <c r="D11" s="5">
         <v>2</v>
       </c>
       <c r="E11" t="s">
@@ -1025,15 +1031,15 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="3">
-        <v>3</v>
-      </c>
-      <c r="D12" s="3">
+      <c r="C12" s="5">
+        <v>3</v>
+      </c>
+      <c r="D12" s="5">
         <v>0</v>
       </c>
       <c r="E12" t="s">
@@ -1045,15 +1051,15 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B13" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="3">
-        <v>2</v>
-      </c>
-      <c r="D13" s="3">
+      <c r="C13" s="5">
+        <v>2</v>
+      </c>
+      <c r="D13" s="5">
         <v>2</v>
       </c>
       <c r="E13" t="s">
@@ -1065,15 +1071,15 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B14" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="5">
         <v>13</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="5">
         <v>1</v>
       </c>
       <c r="E14" t="s">
@@ -1085,15 +1091,15 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B15" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15" s="5">
         <v>14</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="5">
         <v>2</v>
       </c>
       <c r="E15" t="s">
@@ -1105,15 +1111,15 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B16" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="5">
         <v>15</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="5">
         <v>3</v>
       </c>
       <c r="E16" t="s">
@@ -1125,15 +1131,15 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B17" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17" s="5">
         <v>16</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="5">
         <v>1</v>
       </c>
       <c r="E17" t="s">
@@ -1145,15 +1151,15 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B18" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="5">
         <v>17</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="5">
         <v>2</v>
       </c>
       <c r="E18" t="s">
@@ -1165,15 +1171,15 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B19" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19" s="5">
         <v>18</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="5">
         <v>3</v>
       </c>
       <c r="E19" t="s">
@@ -1185,15 +1191,15 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B20" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="5">
         <v>19</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="5">
         <v>1</v>
       </c>
       <c r="E20" t="s">
@@ -1205,15 +1211,15 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B21" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21" s="5">
         <v>20</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="5">
         <v>2</v>
       </c>
       <c r="E21" t="s">
@@ -1225,15 +1231,15 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B22" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C22" s="5">
         <v>21</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="5">
         <v>3</v>
       </c>
       <c r="E22" t="s">
@@ -1245,15 +1251,15 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B23" t="s">
         <v>36</v>
       </c>
-      <c r="C23" s="3">
+      <c r="C23" s="5">
         <v>22</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D23" s="5">
         <v>1</v>
       </c>
       <c r="E23" t="s">
@@ -1265,15 +1271,15 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B24" t="s">
         <v>36</v>
       </c>
-      <c r="C24" s="3">
+      <c r="C24" s="5">
         <v>23</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D24" s="5">
         <v>2</v>
       </c>
       <c r="E24" t="s">
@@ -1285,15 +1291,15 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B25" t="s">
         <v>33</v>
       </c>
-      <c r="C25" s="3">
+      <c r="C25" s="5">
         <v>24</v>
       </c>
-      <c r="D25" s="3">
+      <c r="D25" s="5">
         <v>3</v>
       </c>
       <c r="E25" t="s">
@@ -1305,15 +1311,15 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B26" t="s">
         <v>42</v>
       </c>
-      <c r="C26" s="3">
+      <c r="C26" s="5">
         <v>25</v>
       </c>
-      <c r="D26" s="3">
+      <c r="D26" s="5">
         <v>1</v>
       </c>
       <c r="E26" t="s">
@@ -1325,15 +1331,15 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B27" t="s">
         <v>45</v>
       </c>
-      <c r="C27" s="3">
+      <c r="C27" s="5">
         <v>26</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D27" s="5">
         <v>2</v>
       </c>
       <c r="E27" t="s">
@@ -1345,15 +1351,15 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B28" t="s">
         <v>42</v>
       </c>
-      <c r="C28" s="3">
+      <c r="C28" s="5">
         <v>27</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28" s="5">
         <v>3</v>
       </c>
       <c r="E28" t="s">
@@ -1365,15 +1371,15 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B29" t="s">
         <v>46</v>
       </c>
-      <c r="C29" s="3">
+      <c r="C29" s="5">
         <v>28</v>
       </c>
-      <c r="D29" s="3">
+      <c r="D29" s="5">
         <v>1</v>
       </c>
       <c r="E29" t="s">
@@ -1385,15 +1391,15 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B30" t="s">
         <v>46</v>
       </c>
-      <c r="C30" s="3">
+      <c r="C30" s="5">
         <v>29</v>
       </c>
-      <c r="D30" s="3">
+      <c r="D30" s="5">
         <v>2</v>
       </c>
       <c r="E30" t="s">
@@ -1405,15 +1411,15 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B31" t="s">
         <v>43</v>
       </c>
-      <c r="C31" s="3">
+      <c r="C31" s="5">
         <v>30</v>
       </c>
-      <c r="D31" s="3">
+      <c r="D31" s="5">
         <v>3</v>
       </c>
       <c r="E31" t="s">
@@ -1425,15 +1431,15 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B32" t="s">
         <v>52</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C32" s="5">
         <v>31</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D32" s="5">
         <v>1</v>
       </c>
       <c r="E32" t="s">
@@ -1445,15 +1451,15 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B33" t="s">
         <v>55</v>
       </c>
-      <c r="C33" s="3">
+      <c r="C33" s="5">
         <v>32</v>
       </c>
-      <c r="D33" s="3">
+      <c r="D33" s="5">
         <v>2</v>
       </c>
       <c r="E33" t="s">
@@ -1465,15 +1471,15 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B34" t="s">
         <v>52</v>
       </c>
-      <c r="C34" s="3">
+      <c r="C34" s="5">
         <v>33</v>
       </c>
-      <c r="D34" s="3">
+      <c r="D34" s="5">
         <v>3</v>
       </c>
       <c r="E34" t="s">
@@ -1485,15 +1491,15 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B35" t="s">
         <v>56</v>
       </c>
-      <c r="C35" s="3">
+      <c r="C35" s="5">
         <v>34</v>
       </c>
-      <c r="D35" s="3">
+      <c r="D35" s="5">
         <v>1</v>
       </c>
       <c r="E35" t="s">
@@ -1505,15 +1511,15 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B36" t="s">
         <v>56</v>
       </c>
-      <c r="C36" s="3">
+      <c r="C36" s="5">
         <v>35</v>
       </c>
-      <c r="D36" s="3">
+      <c r="D36" s="5">
         <v>2</v>
       </c>
       <c r="E36" t="s">
@@ -1525,15 +1531,15 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B37" t="s">
         <v>53</v>
       </c>
-      <c r="C37" s="3">
+      <c r="C37" s="5">
         <v>36</v>
       </c>
-      <c r="D37" s="3">
+      <c r="D37" s="5">
         <v>3</v>
       </c>
       <c r="E37" t="s">
@@ -1545,15 +1551,15 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B38" t="s">
         <v>62</v>
       </c>
-      <c r="C38" s="3">
+      <c r="C38" s="5">
         <v>37</v>
       </c>
-      <c r="D38" s="3">
+      <c r="D38" s="5">
         <v>1</v>
       </c>
       <c r="E38" t="s">
@@ -1565,15 +1571,15 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B39" t="s">
         <v>65</v>
       </c>
-      <c r="C39" s="3">
+      <c r="C39" s="5">
         <v>38</v>
       </c>
-      <c r="D39" s="3">
+      <c r="D39" s="5">
         <v>2</v>
       </c>
       <c r="E39" t="s">
@@ -1585,15 +1591,15 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B40" t="s">
         <v>62</v>
       </c>
-      <c r="C40" s="3">
+      <c r="C40" s="5">
         <v>39</v>
       </c>
-      <c r="D40" s="3">
+      <c r="D40" s="5">
         <v>3</v>
       </c>
       <c r="E40" t="s">
@@ -1605,15 +1611,15 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B41" t="s">
         <v>66</v>
       </c>
-      <c r="C41" s="3">
+      <c r="C41" s="5">
         <v>40</v>
       </c>
-      <c r="D41" s="3">
+      <c r="D41" s="5">
         <v>1</v>
       </c>
       <c r="E41" t="s">
@@ -1625,15 +1631,15 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B42" t="s">
         <v>66</v>
       </c>
-      <c r="C42" s="3">
+      <c r="C42" s="5">
         <v>41</v>
       </c>
-      <c r="D42" s="3">
+      <c r="D42" s="5">
         <v>2</v>
       </c>
       <c r="E42" t="s">
@@ -1645,15 +1651,15 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B43" t="s">
         <v>63</v>
       </c>
-      <c r="C43" s="3">
+      <c r="C43" s="5">
         <v>42</v>
       </c>
-      <c r="D43" s="3">
+      <c r="D43" s="5">
         <v>3</v>
       </c>
       <c r="E43" t="s">
@@ -1665,15 +1671,15 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B44" t="s">
         <v>72</v>
       </c>
-      <c r="C44" s="3">
+      <c r="C44" s="5">
         <v>43</v>
       </c>
-      <c r="D44" s="3">
+      <c r="D44" s="5">
         <v>1</v>
       </c>
       <c r="E44" t="s">
@@ -1685,15 +1691,15 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B45" t="s">
         <v>75</v>
       </c>
-      <c r="C45" s="3">
+      <c r="C45" s="5">
         <v>44</v>
       </c>
-      <c r="D45" s="3">
+      <c r="D45" s="5">
         <v>2</v>
       </c>
       <c r="E45" t="s">
@@ -1705,15 +1711,15 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B46" t="s">
         <v>72</v>
       </c>
-      <c r="C46" s="3">
+      <c r="C46" s="5">
         <v>45</v>
       </c>
-      <c r="D46" s="3">
+      <c r="D46" s="5">
         <v>3</v>
       </c>
       <c r="E46" t="s">
@@ -1725,15 +1731,15 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B47" t="s">
         <v>76</v>
       </c>
-      <c r="C47" s="3">
+      <c r="C47" s="5">
         <v>46</v>
       </c>
-      <c r="D47" s="3">
+      <c r="D47" s="5">
         <v>1</v>
       </c>
       <c r="E47" t="s">
@@ -1745,15 +1751,15 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B48" t="s">
         <v>76</v>
       </c>
-      <c r="C48" s="3">
+      <c r="C48" s="5">
         <v>47</v>
       </c>
-      <c r="D48" s="3">
+      <c r="D48" s="5">
         <v>2</v>
       </c>
       <c r="E48" t="s">
@@ -1765,15 +1771,15 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B49" t="s">
         <v>73</v>
       </c>
-      <c r="C49" s="3">
+      <c r="C49" s="5">
         <v>48</v>
       </c>
-      <c r="D49" s="3">
+      <c r="D49" s="5">
         <v>3</v>
       </c>
       <c r="E49" t="s">
@@ -1785,15 +1791,15 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B50" t="s">
         <v>82</v>
       </c>
-      <c r="C50" s="3">
+      <c r="C50" s="5">
         <v>49</v>
       </c>
-      <c r="D50" s="3">
+      <c r="D50" s="5">
         <v>1</v>
       </c>
       <c r="E50" t="s">
@@ -1805,15 +1811,15 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B51" t="s">
         <v>85</v>
       </c>
-      <c r="C51" s="3">
+      <c r="C51" s="5">
         <v>50</v>
       </c>
-      <c r="D51" s="3">
+      <c r="D51" s="5">
         <v>2</v>
       </c>
       <c r="E51" t="s">
@@ -1825,15 +1831,15 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B52" t="s">
         <v>82</v>
       </c>
-      <c r="C52" s="3">
+      <c r="C52" s="5">
         <v>51</v>
       </c>
-      <c r="D52" s="3">
+      <c r="D52" s="5">
         <v>3</v>
       </c>
       <c r="E52" t="s">
@@ -1845,15 +1851,15 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B53" t="s">
         <v>86</v>
       </c>
-      <c r="C53" s="3">
+      <c r="C53" s="5">
         <v>52</v>
       </c>
-      <c r="D53" s="3">
+      <c r="D53" s="5">
         <v>1</v>
       </c>
       <c r="E53" t="s">
@@ -1865,15 +1871,15 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B54" t="s">
         <v>86</v>
       </c>
-      <c r="C54" s="3">
+      <c r="C54" s="5">
         <v>53</v>
       </c>
-      <c r="D54" s="3">
+      <c r="D54" s="5">
         <v>2</v>
       </c>
       <c r="E54" t="s">
@@ -1885,15 +1891,15 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B55" t="s">
         <v>83</v>
       </c>
-      <c r="C55" s="3">
+      <c r="C55" s="5">
         <v>54</v>
       </c>
-      <c r="D55" s="3">
+      <c r="D55" s="5">
         <v>3</v>
       </c>
       <c r="E55" t="s">
@@ -1905,362 +1911,362 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B56" t="s">
         <v>92</v>
       </c>
-      <c r="C56" s="3">
+      <c r="C56" s="5">
         <v>55</v>
       </c>
-      <c r="D56" s="3">
+      <c r="D56" s="5">
         <v>1</v>
       </c>
       <c r="E56" t="s">
+        <v>137</v>
+      </c>
+      <c r="F56" t="s">
         <v>93</v>
-      </c>
-      <c r="F56" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B57" t="s">
+        <v>94</v>
+      </c>
+      <c r="C57" s="5">
+        <v>56</v>
+      </c>
+      <c r="D57" s="5">
+        <v>2</v>
+      </c>
+      <c r="E57" t="s">
         <v>95</v>
       </c>
-      <c r="C57" s="3">
-        <v>56</v>
-      </c>
-      <c r="D57" s="3">
-        <v>2</v>
-      </c>
-      <c r="E57" t="s">
+      <c r="F57" t="s">
         <v>96</v>
-      </c>
-      <c r="F57" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B58" t="s">
         <v>92</v>
       </c>
-      <c r="C58" s="3">
+      <c r="C58" s="5">
         <v>57</v>
       </c>
-      <c r="D58" s="3">
+      <c r="D58" s="5">
         <v>3</v>
       </c>
       <c r="E58" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F58" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B59" t="s">
-        <v>96</v>
-      </c>
-      <c r="C59" s="3">
+        <v>95</v>
+      </c>
+      <c r="C59" s="5">
         <v>58</v>
       </c>
-      <c r="D59" s="3">
+      <c r="D59" s="5">
         <v>1</v>
       </c>
       <c r="E59" t="s">
-        <v>93</v>
+        <v>137</v>
       </c>
       <c r="F59" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B60" t="s">
-        <v>96</v>
-      </c>
-      <c r="C60" s="3">
+        <v>95</v>
+      </c>
+      <c r="C60" s="5">
         <v>59</v>
       </c>
-      <c r="D60" s="3">
+      <c r="D60" s="5">
         <v>2</v>
       </c>
       <c r="E60" t="s">
         <v>92</v>
       </c>
       <c r="F60" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B61" t="s">
-        <v>93</v>
-      </c>
-      <c r="C61" s="3">
+        <v>137</v>
+      </c>
+      <c r="C61" s="5">
         <v>60</v>
       </c>
-      <c r="D61" s="3">
+      <c r="D61" s="5">
         <v>3</v>
       </c>
       <c r="E61" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F61" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B62" t="s">
+        <v>101</v>
+      </c>
+      <c r="C62" s="5">
+        <v>61</v>
+      </c>
+      <c r="D62" s="5">
+        <v>1</v>
+      </c>
+      <c r="E62" t="s">
         <v>102</v>
       </c>
-      <c r="C62" s="3">
-        <v>61</v>
-      </c>
-      <c r="D62" s="3">
-        <v>1</v>
-      </c>
-      <c r="E62" t="s">
+      <c r="F62" t="s">
         <v>103</v>
-      </c>
-      <c r="F62" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B63" t="s">
+        <v>104</v>
+      </c>
+      <c r="C63" s="5">
+        <v>62</v>
+      </c>
+      <c r="D63" s="5">
+        <v>2</v>
+      </c>
+      <c r="E63" t="s">
         <v>105</v>
       </c>
-      <c r="C63" s="3">
-        <v>62</v>
-      </c>
-      <c r="D63" s="3">
-        <v>2</v>
-      </c>
-      <c r="E63" t="s">
+      <c r="F63" t="s">
         <v>106</v>
-      </c>
-      <c r="F63" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B64" t="s">
-        <v>102</v>
-      </c>
-      <c r="C64" s="3">
+        <v>101</v>
+      </c>
+      <c r="C64" s="5">
         <v>63</v>
       </c>
-      <c r="D64" s="3">
+      <c r="D64" s="5">
         <v>3</v>
       </c>
       <c r="E64" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F64" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B65" t="s">
-        <v>106</v>
-      </c>
-      <c r="C65" s="3">
+        <v>105</v>
+      </c>
+      <c r="C65" s="5">
         <v>64</v>
       </c>
-      <c r="D65" s="3">
+      <c r="D65" s="5">
         <v>1</v>
       </c>
       <c r="E65" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F65" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B66" t="s">
-        <v>106</v>
-      </c>
-      <c r="C66" s="3">
+        <v>105</v>
+      </c>
+      <c r="C66" s="5">
         <v>65</v>
       </c>
-      <c r="D66" s="3">
+      <c r="D66" s="5">
         <v>2</v>
       </c>
       <c r="E66" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F66" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B67" t="s">
-        <v>103</v>
-      </c>
-      <c r="C67" s="3">
+        <v>102</v>
+      </c>
+      <c r="C67" s="5">
         <v>66</v>
       </c>
-      <c r="D67" s="3">
+      <c r="D67" s="5">
         <v>3</v>
       </c>
       <c r="E67" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F67" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B68" t="s">
+        <v>111</v>
+      </c>
+      <c r="C68" s="5">
+        <v>67</v>
+      </c>
+      <c r="D68" s="5">
+        <v>1</v>
+      </c>
+      <c r="E68" t="s">
         <v>112</v>
       </c>
-      <c r="C68" s="3">
-        <v>67</v>
-      </c>
-      <c r="D68" s="3">
-        <v>1</v>
-      </c>
-      <c r="E68" t="s">
+      <c r="F68" t="s">
         <v>113</v>
-      </c>
-      <c r="F68" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B69" t="s">
+        <v>114</v>
+      </c>
+      <c r="C69" s="5">
+        <v>68</v>
+      </c>
+      <c r="D69" s="5">
+        <v>2</v>
+      </c>
+      <c r="E69" t="s">
         <v>115</v>
       </c>
-      <c r="C69" s="3">
-        <v>68</v>
-      </c>
-      <c r="D69" s="3">
-        <v>2</v>
-      </c>
-      <c r="E69" t="s">
+      <c r="F69" t="s">
         <v>116</v>
-      </c>
-      <c r="F69" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B70" t="s">
-        <v>112</v>
-      </c>
-      <c r="C70" s="3">
+        <v>111</v>
+      </c>
+      <c r="C70" s="5">
         <v>69</v>
       </c>
-      <c r="D70" s="3">
+      <c r="D70" s="5">
         <v>3</v>
       </c>
       <c r="E70" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F70" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B71" t="s">
-        <v>116</v>
-      </c>
-      <c r="C71" s="3">
+        <v>115</v>
+      </c>
+      <c r="C71" s="5">
         <v>70</v>
       </c>
-      <c r="D71" s="3">
+      <c r="D71" s="5">
         <v>1</v>
       </c>
       <c r="E71" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F71" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B72" t="s">
-        <v>116</v>
-      </c>
-      <c r="C72" s="3">
+        <v>115</v>
+      </c>
+      <c r="C72" s="5">
         <v>71</v>
       </c>
-      <c r="D72" s="3">
+      <c r="D72" s="5">
         <v>2</v>
       </c>
       <c r="E72" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F72" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B73" t="s">
-        <v>113</v>
-      </c>
-      <c r="C73" s="3">
+        <v>112</v>
+      </c>
+      <c r="C73" s="5">
         <v>72</v>
       </c>
-      <c r="D73" s="3">
+      <c r="D73" s="5">
         <v>3</v>
       </c>
       <c r="E73" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F73" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
minor correction + folder cleaning
</commit_message>
<xml_diff>
--- a/runapp/www/scores.xlsx
+++ b/runapp/www/scores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loicl\OneDrive\Documents\Loïc\Divers_non_disque\Data_science\Projet\MesProjets\Coupe_du_monde_2026\runapp\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{519303FB-C163-4C23-A7B5-8BC63AAC1E8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9186B043-0127-444E-BFA2-7D0135404506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -863,12 +863,6 @@
       <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
       <c r="F2" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Time optimized + UI enhanced
</commit_message>
<xml_diff>
--- a/runapp/www/scores.xlsx
+++ b/runapp/www/scores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loicl\OneDrive\Documents\Loïc\Divers_non_disque\Data_science\Projet\MesProjets\Coupe_du_monde_2026\runapp\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9186B043-0127-444E-BFA2-7D0135404506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4087C56B-0379-47F3-B0AA-4FF75A03273F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5760" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="137">
   <si>
     <t>Group</t>
   </si>
@@ -341,9 +341,6 @@
   </si>
   <si>
     <t>66456928</t>
-  </si>
-  <si>
-    <t>66456934</t>
   </si>
   <si>
     <t>66456912</t>
@@ -523,7 +520,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B5B661F2-F11D-4CF0-A27D-C7750D0CA641}" name="Tableau1" displayName="Tableau1" ref="A1:F73" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:F73" xr:uid="{B5B661F2-F11D-4CF0-A27D-C7750D0CA641}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F73">
-    <sortCondition ref="B1:B73"/>
+    <sortCondition ref="A1:A73"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{F30B2D7B-C281-4804-AE2F-1FE4286D5F6E}" name="Group"/>
@@ -828,9 +825,10 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.77734375" customWidth="1"/>
-    <col min="3" max="3" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.5546875" customWidth="1"/>
     <col min="5" max="5" width="13.21875" customWidth="1"/>
+    <col min="6" max="6" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -863,6 +861,12 @@
       <c r="C2" t="s">
         <v>8</v>
       </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
       <c r="F2" t="s">
         <v>9</v>
       </c>
@@ -872,10 +876,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C3" t="s">
-        <v>126</v>
+        <v>125</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
       </c>
       <c r="F3" t="s">
         <v>11</v>
@@ -886,13 +896,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
       </c>
       <c r="F4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -914,7 +924,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
@@ -928,13 +938,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C7" t="s">
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -947,6 +957,12 @@
       <c r="C8" t="s">
         <v>51</v>
       </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
       <c r="F8" t="s">
         <v>49</v>
       </c>
@@ -956,10 +972,16 @@
         <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C9" t="s">
-        <v>121</v>
+        <v>120</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
       </c>
       <c r="F9" t="s">
         <v>48</v>
@@ -970,13 +992,13 @@
         <v>46</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C10" t="s">
         <v>51</v>
       </c>
       <c r="F10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1012,13 +1034,13 @@
         <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C13" t="s">
         <v>49</v>
       </c>
       <c r="F13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -1031,6 +1053,12 @@
       <c r="C14" t="s">
         <v>55</v>
       </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
       <c r="F14" t="s">
         <v>91</v>
       </c>
@@ -1045,6 +1073,12 @@
       <c r="C15" t="s">
         <v>74</v>
       </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
       <c r="F15" t="s">
         <v>54</v>
       </c>
@@ -1067,8 +1101,8 @@
       <c r="A17" t="s">
         <v>52</v>
       </c>
-      <c r="B17" t="s">
-        <v>107</v>
+      <c r="B17">
+        <v>66456934</v>
       </c>
       <c r="C17" t="s">
         <v>54</v>
@@ -1110,10 +1144,16 @@
         <v>33</v>
       </c>
       <c r="B20" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C20" t="s">
         <v>38</v>
+      </c>
+      <c r="D20">
+        <v>4</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
       </c>
       <c r="F20" t="s">
         <v>35</v>
@@ -1124,10 +1164,16 @@
         <v>33</v>
       </c>
       <c r="B21" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C21" t="s">
         <v>36</v>
+      </c>
+      <c r="D21">
+        <v>2</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
       </c>
       <c r="F21" t="s">
         <v>81</v>
@@ -1152,7 +1198,7 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C23" t="s">
         <v>81</v>
@@ -1191,674 +1237,704 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>99</v>
+        <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="C26" t="s">
-        <v>101</v>
+        <v>21</v>
+      </c>
+      <c r="D26">
+        <v>7</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>102</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>99</v>
+        <v>18</v>
       </c>
       <c r="B27" t="s">
-        <v>135</v>
+        <v>78</v>
       </c>
       <c r="C27" t="s">
-        <v>132</v>
+        <v>65</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
       </c>
       <c r="F27" t="s">
-        <v>104</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>99</v>
+        <v>18</v>
       </c>
       <c r="B28" t="s">
-        <v>133</v>
+        <v>64</v>
       </c>
       <c r="C28" t="s">
-        <v>101</v>
+        <v>21</v>
       </c>
       <c r="F28" t="s">
-        <v>132</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>99</v>
+        <v>18</v>
       </c>
       <c r="B29" t="s">
-        <v>103</v>
+        <v>72</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
+        <v>20</v>
       </c>
       <c r="F29" t="s">
-        <v>102</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>99</v>
+        <v>18</v>
       </c>
       <c r="B30" t="s">
-        <v>118</v>
+        <v>19</v>
       </c>
       <c r="C30" t="s">
-        <v>104</v>
+        <v>20</v>
       </c>
       <c r="F30" t="s">
-        <v>101</v>
+        <v>21</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>99</v>
+        <v>18</v>
       </c>
       <c r="B31" t="s">
-        <v>131</v>
+        <v>66</v>
       </c>
       <c r="C31" t="s">
-        <v>102</v>
+        <v>67</v>
       </c>
       <c r="F31" t="s">
-        <v>132</v>
+        <v>65</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>42</v>
+        <v>99</v>
       </c>
       <c r="B32" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C32" t="s">
-        <v>45</v>
+        <v>101</v>
+      </c>
+      <c r="D32">
+        <v>2</v>
+      </c>
+      <c r="E32">
+        <v>2</v>
       </c>
       <c r="F32" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>42</v>
+        <v>99</v>
       </c>
       <c r="B33" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="C33" t="s">
-        <v>97</v>
+        <v>131</v>
+      </c>
+      <c r="D33">
+        <v>5</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>44</v>
+        <v>104</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>42</v>
+        <v>99</v>
       </c>
       <c r="B34" t="s">
-        <v>96</v>
+        <v>132</v>
       </c>
       <c r="C34" t="s">
-        <v>45</v>
+        <v>101</v>
       </c>
       <c r="F34" t="s">
-        <v>97</v>
+        <v>131</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>42</v>
+        <v>99</v>
       </c>
       <c r="B35" t="s">
-        <v>77</v>
+        <v>103</v>
       </c>
       <c r="C35" t="s">
-        <v>44</v>
+        <v>104</v>
       </c>
       <c r="F35" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>42</v>
+        <v>99</v>
       </c>
       <c r="B36" t="s">
-        <v>43</v>
+        <v>117</v>
       </c>
       <c r="C36" t="s">
-        <v>44</v>
+        <v>104</v>
       </c>
       <c r="F36" t="s">
-        <v>45</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>42</v>
+        <v>99</v>
       </c>
       <c r="B37" t="s">
-        <v>98</v>
+        <v>130</v>
       </c>
       <c r="C37" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="F37" t="s">
-        <v>97</v>
+        <v>131</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="B38" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="C38" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="F38" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="B39" t="s">
-        <v>137</v>
+        <v>109</v>
       </c>
       <c r="C39" t="s">
-        <v>29</v>
+        <v>97</v>
       </c>
       <c r="F39" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="B40" t="s">
-        <v>30</v>
+        <v>96</v>
       </c>
       <c r="C40" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="F40" t="s">
-        <v>29</v>
+        <v>97</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="B41" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="C41" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="F41" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="B42" t="s">
-        <v>79</v>
+        <v>43</v>
       </c>
       <c r="C42" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="F42" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="C43" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="F43" t="s">
-        <v>29</v>
+        <v>97</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="B44" t="s">
-        <v>129</v>
+        <v>57</v>
       </c>
       <c r="C44" t="s">
-        <v>85</v>
+        <v>31</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
       </c>
       <c r="F44" t="s">
-        <v>95</v>
+        <v>28</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="B45" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="C45" t="s">
-        <v>93</v>
+        <v>29</v>
       </c>
       <c r="F45" t="s">
-        <v>84</v>
+        <v>59</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="B46" t="s">
-        <v>92</v>
+        <v>30</v>
       </c>
       <c r="C46" t="s">
-        <v>85</v>
+        <v>31</v>
       </c>
       <c r="F46" t="s">
-        <v>93</v>
+        <v>29</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="B47" t="s">
-        <v>130</v>
+        <v>58</v>
       </c>
       <c r="C47" t="s">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="F47" t="s">
-        <v>95</v>
+        <v>28</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="B48" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C48" t="s">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="F48" t="s">
-        <v>85</v>
+        <v>31</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="B49" t="s">
-        <v>94</v>
+        <v>27</v>
       </c>
       <c r="C49" t="s">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="F49" t="s">
-        <v>93</v>
+        <v>29</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="B50" t="s">
-        <v>13</v>
+        <v>128</v>
       </c>
       <c r="C50" t="s">
-        <v>14</v>
+        <v>85</v>
       </c>
       <c r="F50" t="s">
-        <v>15</v>
+        <v>95</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="B51" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C51" t="s">
-        <v>40</v>
+        <v>93</v>
       </c>
       <c r="F51" t="s">
-        <v>17</v>
+        <v>84</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="B52" t="s">
-        <v>39</v>
+        <v>92</v>
       </c>
       <c r="C52" t="s">
-        <v>14</v>
+        <v>85</v>
       </c>
       <c r="F52" t="s">
-        <v>40</v>
+        <v>93</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="B53" t="s">
-        <v>16</v>
+        <v>129</v>
       </c>
       <c r="C53" t="s">
-        <v>17</v>
+        <v>84</v>
       </c>
       <c r="F53" t="s">
-        <v>15</v>
+        <v>95</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="B54" t="s">
-        <v>32</v>
+        <v>83</v>
       </c>
       <c r="C54" t="s">
-        <v>17</v>
+        <v>84</v>
       </c>
       <c r="F54" t="s">
-        <v>14</v>
+        <v>85</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="B55" t="s">
-        <v>41</v>
+        <v>94</v>
       </c>
       <c r="C55" t="s">
-        <v>15</v>
+        <v>95</v>
       </c>
       <c r="F55" t="s">
-        <v>40</v>
+        <v>93</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="C56" t="s">
-        <v>114</v>
+        <v>14</v>
       </c>
       <c r="F56" t="s">
-        <v>112</v>
+        <v>15</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>61</v>
+        <v>105</v>
       </c>
       <c r="C57" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="F57" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>113</v>
+        <v>39</v>
       </c>
       <c r="C58" t="s">
-        <v>114</v>
+        <v>14</v>
       </c>
       <c r="F58" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="B59" t="s">
-        <v>123</v>
+        <v>16</v>
       </c>
       <c r="C59" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
       <c r="F59" t="s">
-        <v>112</v>
+        <v>15</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="B60" t="s">
-        <v>119</v>
+        <v>32</v>
       </c>
       <c r="C60" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
       <c r="F60" t="s">
-        <v>114</v>
+        <v>14</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="B61" t="s">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="C61" t="s">
-        <v>112</v>
+        <v>15</v>
       </c>
       <c r="F61" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="C62" t="s">
-        <v>25</v>
+        <v>113</v>
       </c>
       <c r="F62" t="s">
-        <v>69</v>
+        <v>111</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="B63" t="s">
-        <v>115</v>
+        <v>61</v>
       </c>
       <c r="C63" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="F63" t="s">
-        <v>24</v>
+        <v>63</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="B64" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="C64" t="s">
-        <v>25</v>
+        <v>113</v>
       </c>
       <c r="F64" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="B65" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="C65" t="s">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="F65" t="s">
-        <v>69</v>
+        <v>111</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="B66" t="s">
-        <v>23</v>
+        <v>118</v>
       </c>
       <c r="C66" t="s">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="F66" t="s">
-        <v>25</v>
+        <v>113</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="B67" t="s">
-        <v>86</v>
+        <v>110</v>
       </c>
       <c r="C67" t="s">
-        <v>69</v>
+        <v>111</v>
       </c>
       <c r="F67" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B68" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C68" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F68" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B69" t="s">
-        <v>78</v>
+        <v>114</v>
       </c>
       <c r="C69" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="F69" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B70" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="C70" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F70" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B71" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C71" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F71" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B72" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C72" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F72" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B73" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="C73" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F73" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update ui + proba
</commit_message>
<xml_diff>
--- a/runapp/www/scores.xlsx
+++ b/runapp/www/scores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loicl\OneDrive\Documents\Loïc\Divers_non_disque\Data_science\Projet\MesProjets\Coupe_du_monde_2026\runapp\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4087C56B-0379-47F3-B0AA-4FF75A03273F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49A99EE9-CFCE-4CD4-9900-A4E9EC113144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1437,6 +1437,12 @@
       <c r="C38" t="s">
         <v>45</v>
       </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
       <c r="F38" t="s">
         <v>76</v>
       </c>
@@ -1451,6 +1457,12 @@
       <c r="C39" t="s">
         <v>97</v>
       </c>
+      <c r="D39">
+        <v>2</v>
+      </c>
+      <c r="E39">
+        <v>2</v>
+      </c>
       <c r="F39" t="s">
         <v>44</v>
       </c>
@@ -1541,6 +1553,12 @@
       <c r="C45" t="s">
         <v>29</v>
       </c>
+      <c r="D45">
+        <v>1</v>
+      </c>
+      <c r="E45">
+        <v>1</v>
+      </c>
       <c r="F45" t="s">
         <v>59</v>
       </c>
@@ -1611,6 +1629,12 @@
       <c r="C50" t="s">
         <v>85</v>
       </c>
+      <c r="D50">
+        <v>3</v>
+      </c>
+      <c r="E50">
+        <v>1</v>
+      </c>
       <c r="F50" t="s">
         <v>95</v>
       </c>
@@ -1625,6 +1649,12 @@
       <c r="C51" t="s">
         <v>93</v>
       </c>
+      <c r="D51">
+        <v>1</v>
+      </c>
+      <c r="E51">
+        <v>4</v>
+      </c>
       <c r="F51" t="s">
         <v>84</v>
       </c>
@@ -1695,6 +1725,12 @@
       <c r="C56" t="s">
         <v>14</v>
       </c>
+      <c r="D56">
+        <v>3</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
       <c r="F56" t="s">
         <v>15</v>
       </c>
@@ -1708,6 +1744,12 @@
       </c>
       <c r="C57" t="s">
         <v>40</v>
+      </c>
+      <c r="D57">
+        <v>3</v>
+      </c>
+      <c r="E57">
+        <v>1</v>
       </c>
       <c r="F57" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
scores & proba update
</commit_message>
<xml_diff>
--- a/runapp/www/scores.xlsx
+++ b/runapp/www/scores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loicl\OneDrive\Documents\Loïc\Divers_non_disque\Data_science\Projet\MesProjets\Coupe_du_monde_2026\runapp\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B272D1-A109-479E-9DAD-353EDCE400FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68AAB3F0-0784-4D1F-A6D2-4B65B14C4097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1117,6 +1117,12 @@
       <c r="C16" t="s">
         <v>55</v>
       </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
       <c r="F16" t="s">
         <v>74</v>
       </c>
@@ -1131,6 +1137,12 @@
       <c r="C17" t="s">
         <v>54</v>
       </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
       <c r="F17" t="s">
         <v>91</v>
       </c>
@@ -1213,6 +1225,12 @@
       <c r="C22" t="s">
         <v>38</v>
       </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
       <c r="F22" t="s">
         <v>36</v>
       </c>
@@ -1227,6 +1245,12 @@
       <c r="C23" t="s">
         <v>81</v>
       </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
       <c r="F23" t="s">
         <v>35</v>
       </c>
@@ -1309,6 +1333,12 @@
       <c r="C28" t="s">
         <v>21</v>
       </c>
+      <c r="D28">
+        <v>2</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
       <c r="F28" t="s">
         <v>65</v>
       </c>
@@ -1323,6 +1353,12 @@
       <c r="C29" t="s">
         <v>20</v>
       </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
       <c r="F29" t="s">
         <v>67</v>
       </c>
@@ -1405,6 +1441,12 @@
       <c r="C34" t="s">
         <v>101</v>
       </c>
+      <c r="D34">
+        <v>5</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
       <c r="F34" t="s">
         <v>131</v>
       </c>
@@ -1418,6 +1460,12 @@
       </c>
       <c r="C35" t="s">
         <v>104</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>4</v>
       </c>
       <c r="F35" t="s">
         <v>102</v>

</xml_diff>

<commit_message>
correct 1 tab + update score and proba
</commit_message>
<xml_diff>
--- a/runapp/www/scores.xlsx
+++ b/runapp/www/scores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loicl\OneDrive\Documents\Loïc\Divers_non_disque\Data_science\Projet\MesProjets\Coupe_du_monde_2026\runapp\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68AAB3F0-0784-4D1F-A6D2-4B65B14C4097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F93963D-83B9-4DCC-9DF2-2AD36D7933C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1549,6 +1549,12 @@
       <c r="C40" t="s">
         <v>45</v>
       </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
       <c r="F40" t="s">
         <v>97</v>
       </c>
@@ -1563,6 +1569,12 @@
       <c r="C41" t="s">
         <v>44</v>
       </c>
+      <c r="D41">
+        <v>1</v>
+      </c>
+      <c r="E41">
+        <v>3</v>
+      </c>
       <c r="F41" t="s">
         <v>76</v>
       </c>
@@ -1645,6 +1657,12 @@
       <c r="C46" t="s">
         <v>31</v>
       </c>
+      <c r="D46">
+        <v>4</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
       <c r="F46" t="s">
         <v>29</v>
       </c>
@@ -1658,6 +1676,12 @@
       </c>
       <c r="C47" t="s">
         <v>59</v>
+      </c>
+      <c r="D47">
+        <v>2</v>
+      </c>
+      <c r="E47">
+        <v>2</v>
       </c>
       <c r="F47" t="s">
         <v>28</v>

</xml_diff>